<commit_message>
atualização do resultado e a forma de apresentar os resultados
</commit_message>
<xml_diff>
--- a/resultados/Grade_Horarios_CADASTRO_TURMAS_20262.xlsx
+++ b/resultados/Grade_Horarios_CADASTRO_TURMAS_20262.xlsx
@@ -151,8 +151,8 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="Legenda_Fase_5" displayName="Legenda_Fase_5" ref="A19:D24" headerRowCount="1">
-  <autoFilter ref="A19:D24"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="Legenda_Fase_5" displayName="Legenda_Fase_5" ref="A19:D29" headerRowCount="1">
+  <autoFilter ref="A19:D29"/>
   <tableColumns count="4">
     <tableColumn id="1" name="Cód. (Turma)"/>
     <tableColumn id="2" name="Nome da Disciplina"/>
@@ -179,8 +179,8 @@
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="Legenda_Fase_6" displayName="Legenda_Fase_6" ref="A19:D23" headerRowCount="1">
-  <autoFilter ref="A19:D23"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="Legenda_Fase_6" displayName="Legenda_Fase_6" ref="A19:D26" headerRowCount="1">
+  <autoFilter ref="A19:D26"/>
   <tableColumns count="4">
     <tableColumn id="1" name="Cód. (Turma)"/>
     <tableColumn id="2" name="Nome da Disciplina"/>
@@ -592,7 +592,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K67"/>
+  <dimension ref="A1:K64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3069,7 +3069,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Optativa</t>
+          <t>5ª Fase (Optativa)</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -3126,7 +3126,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Optativa</t>
+          <t>5ª Fase (Optativa)</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -3183,7 +3183,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Optativa</t>
+          <t>6ª Fase (Optativa)</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -3282,29 +3282,29 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>CIN7913</t>
+          <t>CIN7917</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>04342</t>
+          <t>05342</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Lógica Instrumental II [Cancelada]</t>
+          <t>Visualização da Informação</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
+          <t>5ª Fase (Optativa)</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
           <t>Optativa</t>
         </is>
       </c>
-      <c r="F48" t="inlineStr">
-        <is>
-          <t>Optativa</t>
-        </is>
-      </c>
       <c r="G48" t="inlineStr">
         <is>
           <t>36</t>
@@ -3312,22 +3312,22 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>26</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>4.1830-2</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>AUX-ALOCAR</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>Disciplina Cancelada</t>
+          <t>Márcio Matias</t>
         </is>
       </c>
     </row>
@@ -3339,27 +3339,27 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>CIN7917</t>
+          <t>CIN7925</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>05342</t>
+          <t>01342</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Visualização da Informação</t>
+          <t>Introdução a Algoritmos</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Optativa</t>
+          <t>1ª Fase</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Optativa</t>
+          <t>Obrigatória</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -3374,7 +3374,7 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>4.1830-2</t>
+          <t>5.2020-2</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
@@ -3384,7 +3384,7 @@
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>Márcio Matias</t>
+          <t>Ricardo Alexandre Reinaldo de Moraes</t>
         </is>
       </c>
     </row>
@@ -3396,17 +3396,17 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>CIN7917</t>
+          <t>CIN7927</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>06342</t>
+          <t>05342</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Visualização da Informação [Cancelada]</t>
+          <t>Gestão da Informação Pública</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -3426,22 +3426,22 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>26</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>2.1830-2</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>AUX-ALOCAR</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>Disciplina Cancelada</t>
+          <t>Sabrina Borges Ramos de Carvalho</t>
         </is>
       </c>
     </row>
@@ -3453,27 +3453,27 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>CIN7925</t>
+          <t>CIN7935</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>01342</t>
+          <t>06342</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Introdução a Algoritmos</t>
+          <t>Liderança e Gerência</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>1ª Fase</t>
+          <t>6ª Fase (Optativa)</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Obrigatória</t>
+          <t>Optativa</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -3488,17 +3488,17 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>5.2020-2</t>
+          <t>5.1830-2</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>AUX-ALOCAR</t>
+          <t>CED-LBCON</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>Ricardo Alexandre Reinaldo de Moraes</t>
+          <t>Sonali Paula Molin Bedin</t>
         </is>
       </c>
     </row>
@@ -3510,27 +3510,27 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>CIN7927</t>
+          <t>CIN7936</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>05342</t>
+          <t>03342A</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Gestão da Informação Pública</t>
+          <t>Proteção de Dados Pessoais</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Optativa</t>
+          <t>3ª Fase</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Optativa</t>
+          <t>Obrigatória</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -3540,22 +3540,22 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>2.1830-2</t>
+          <t>2.0820-2</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>AUX-ALOCAR</t>
+          <t>CED-LBPREV</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>Sabrina Borges Ramos de Carvalho</t>
+          <t>Marcelo Minghelli</t>
         </is>
       </c>
     </row>
@@ -3567,27 +3567,27 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>CIN7935</t>
+          <t>CIN7936</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>06342</t>
+          <t>03342C</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Liderança e Gerência</t>
+          <t>Proteção de Dados Pessoais</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Optativa</t>
+          <t>3ª Fase</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Optativa</t>
+          <t>Obrigatória</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -3597,22 +3597,22 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>5.1830-2</t>
+          <t>3.1830-2</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>CED-LBCON</t>
+          <t>CED-102 C</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>Sonali Paula Molin Bedin</t>
+          <t>Marcelo Minghelli</t>
         </is>
       </c>
     </row>
@@ -3624,27 +3624,27 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>CIN7936</t>
+          <t>CIN7938</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>03342A</t>
+          <t>05342</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Proteção de Dados Pessoais</t>
+          <t>Segurança da Informação</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>3ª Fase</t>
+          <t>5ª Fase (Optativa)</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Obrigatória</t>
+          <t>Optativa</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -3654,22 +3654,22 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>30</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>2.0820-2</t>
+          <t>3.2020-2</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>CED-LBPREV</t>
+          <t>AUX-ALOCAR</t>
         </is>
       </c>
       <c r="K54" t="inlineStr">
         <is>
-          <t>Marcelo Minghelli</t>
+          <t>A contratar</t>
         </is>
       </c>
     </row>
@@ -3681,22 +3681,22 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>CIN7936</t>
+          <t>CIN7943</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>03342C</t>
+          <t>01342</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Proteção de Dados Pessoais</t>
+          <t>Experiência do Usuário (UX) User Experience</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>3ª Fase</t>
+          <t>1ª Fase</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -3711,22 +3711,22 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>26</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>3.1830-2</t>
+          <t>4.2020-2</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>CED-102 C</t>
+          <t>AUX-ALOCAR</t>
         </is>
       </c>
       <c r="K55" t="inlineStr">
         <is>
-          <t>Marcelo Minghelli</t>
+          <t>Márcio Matias</t>
         </is>
       </c>
     </row>
@@ -3738,7 +3738,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>CIN7938</t>
+          <t>CIN7945</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -3748,19 +3748,19 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Segurança da Informação</t>
+          <t>Fontes de Informação Tecnológica</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
+          <t>5ª Fase (Optativa)</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
           <t>Optativa</t>
         </is>
       </c>
-      <c r="F56" t="inlineStr">
-        <is>
-          <t>Optativa</t>
-        </is>
-      </c>
       <c r="G56" t="inlineStr">
         <is>
           <t>36</t>
@@ -3768,12 +3768,12 @@
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>26</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>3.2020-2</t>
+          <t>2.2020-2</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
@@ -3783,7 +3783,7 @@
       </c>
       <c r="K56" t="inlineStr">
         <is>
-          <t>A contratar</t>
+          <t>Márcio Matias</t>
         </is>
       </c>
     </row>
@@ -3795,27 +3795,27 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>CIN7943</t>
+          <t>CIN7946</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>01342</t>
+          <t>05342</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Experiência do Usuário (UX) User Experience</t>
+          <t>Pitch de Carreira</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>1ª Fase</t>
+          <t>6ª Fase (Optativa)</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Obrigatória</t>
+          <t>Optativa</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -3830,17 +3830,17 @@
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>4.2020-2</t>
+          <t>5.2020-2</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>AUX-ALOCAR</t>
+          <t>CED-LBCON</t>
         </is>
       </c>
       <c r="K57" t="inlineStr">
         <is>
-          <t>Márcio Matias</t>
+          <t>Sonali Paula Molin Bedin</t>
         </is>
       </c>
     </row>
@@ -3852,52 +3852,52 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>CIN7945</t>
+          <t>HST7921</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>05342</t>
+          <t>03342A</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Fontes de Informação Tecnológica</t>
+          <t>História do Brasil Contemporâneo</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Optativa</t>
+          <t>3ª Fase</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Optativa</t>
+          <t>Obrigatória</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>72</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>2.2020-2</t>
+          <t>5.0820-4</t>
         </is>
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>AUX-ALOCAR</t>
+          <t>CED-LBPREV</t>
         </is>
       </c>
       <c r="K58" t="inlineStr">
         <is>
-          <t>Márcio Matias</t>
+          <t>Roselane Neckel</t>
         </is>
       </c>
     </row>
@@ -3909,52 +3909,52 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>CIN7946</t>
+          <t>HST7921</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>05342</t>
+          <t>03342C</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Pitch de Carreira</t>
+          <t>História do Brasil Contemporâneo</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Optativa</t>
+          <t>3ª Fase</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Optativa</t>
+          <t>Obrigatória</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>72</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>5.2020-2</t>
+          <t>6.1830-4</t>
         </is>
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>CED-LBCON</t>
+          <t>CED-LBPREV</t>
         </is>
       </c>
       <c r="K59" t="inlineStr">
         <is>
-          <t>Sonali Paula Molin Bedin</t>
+          <t>Roselane Neckel</t>
         </is>
       </c>
     </row>
@@ -3966,52 +3966,52 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>CIN7950</t>
+          <t>INE5111</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>06342</t>
+          <t>02342A</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Programa de Intercâmbio I</t>
+          <t>Estatística Aplicada I</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Optativa</t>
+          <t>2ª Fase</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Optativa</t>
+          <t>Obrigatória</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>72</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>24</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>A definir</t>
+          <t>3.0820-2 | 4.1010-2</t>
         </is>
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>A definir</t>
+          <t>CED-LBPREV | CED-LBPREV</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
         <is>
-          <t>A contratar</t>
+          <t>Vera do Carmo Comparsi de Vargas</t>
         </is>
       </c>
     </row>
@@ -4023,22 +4023,22 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>HST7921</t>
+          <t>INE5111</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>03342A</t>
+          <t>02342C</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>História do Brasil Contemporâneo</t>
+          <t>Estatística Aplicada I</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>3ª Fase</t>
+          <t>2ª Fase</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -4053,22 +4053,22 @@
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>24</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>5.0820-4</t>
+          <t>2.1830-2 | 5.1830-2</t>
         </is>
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>CED-LBPREV</t>
+          <t>CED-LBPREV | CED-102 C</t>
         </is>
       </c>
       <c r="K61" t="inlineStr">
         <is>
-          <t>Roselane Neckel</t>
+          <t>Manoella Reis Cardenuto</t>
         </is>
       </c>
     </row>
@@ -4080,22 +4080,22 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>HST7921</t>
+          <t>LLV7802</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>03342C</t>
+          <t>01342C</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>História do Brasil Contemporâneo</t>
+          <t>Leitura e Produção do Texto</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>3ª Fase</t>
+          <t>1ª Fase</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -4120,12 +4120,12 @@
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>CED-LBPREV</t>
+          <t>AUX-ALOCAR</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
         <is>
-          <t>Roselane Neckel</t>
+          <t>Gabriela Rempel</t>
         </is>
       </c>
     </row>
@@ -4137,22 +4137,22 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>INE5111</t>
+          <t>LLV7802</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>02342A</t>
+          <t>01342D</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Estatística Aplicada I</t>
+          <t>Leitura e Produção do Texto</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>2ª Fase</t>
+          <t>1ª Fase</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -4167,22 +4167,22 @@
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>3.0820-2 | 4.1010-2</t>
+          <t>6.1830-4</t>
         </is>
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>CED-LBPREV | CED-LBPREV</t>
+          <t>AUX-ALOCAR</t>
         </is>
       </c>
       <c r="K63" t="inlineStr">
         <is>
-          <t>Vera do Carmo Comparsi de Vargas</t>
+          <t>Silvia Ines Coneglian Carrilho de Vasconcelos</t>
         </is>
       </c>
     </row>
@@ -4194,22 +4194,22 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>INE5111</t>
+          <t>MTM3110</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>02342C</t>
+          <t>01342</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Estatística Aplicada I</t>
+          <t>Cálculo</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>2ª Fase</t>
+          <t>1ª Fase</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
@@ -4219,196 +4219,25 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
           <t>72</t>
         </is>
       </c>
-      <c r="H64" t="inlineStr">
-        <is>
-          <t>24</t>
-        </is>
-      </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>2.1830-2 | 5.1830-2</t>
+          <t>3.1830-2 | 5.1830-2</t>
         </is>
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>CED-LBPREV | CED-102 C</t>
+          <t>AUX-ALOCAR | AUX-ALOCAR</t>
         </is>
       </c>
       <c r="K64" t="inlineStr">
-        <is>
-          <t>Manoella Reis Cardenuto</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>2026.2</t>
-        </is>
-      </c>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t>LLV7802</t>
-        </is>
-      </c>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t>01342C</t>
-        </is>
-      </c>
-      <c r="D65" t="inlineStr">
-        <is>
-          <t>Leitura e Produção do Texto</t>
-        </is>
-      </c>
-      <c r="E65" t="inlineStr">
-        <is>
-          <t>1ª Fase</t>
-        </is>
-      </c>
-      <c r="F65" t="inlineStr">
-        <is>
-          <t>Obrigatória</t>
-        </is>
-      </c>
-      <c r="G65" t="inlineStr">
-        <is>
-          <t>72</t>
-        </is>
-      </c>
-      <c r="H65" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="I65" t="inlineStr">
-        <is>
-          <t>6.1830-4</t>
-        </is>
-      </c>
-      <c r="J65" t="inlineStr">
-        <is>
-          <t>AUX-ALOCAR</t>
-        </is>
-      </c>
-      <c r="K65" t="inlineStr">
-        <is>
-          <t>Gabriela Rempel</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>2026.2</t>
-        </is>
-      </c>
-      <c r="B66" t="inlineStr">
-        <is>
-          <t>LLV7802</t>
-        </is>
-      </c>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t>01342D</t>
-        </is>
-      </c>
-      <c r="D66" t="inlineStr">
-        <is>
-          <t>Leitura e Produção do Texto</t>
-        </is>
-      </c>
-      <c r="E66" t="inlineStr">
-        <is>
-          <t>1ª Fase</t>
-        </is>
-      </c>
-      <c r="F66" t="inlineStr">
-        <is>
-          <t>Obrigatória</t>
-        </is>
-      </c>
-      <c r="G66" t="inlineStr">
-        <is>
-          <t>72</t>
-        </is>
-      </c>
-      <c r="H66" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="I66" t="inlineStr">
-        <is>
-          <t>6.1830-4</t>
-        </is>
-      </c>
-      <c r="J66" t="inlineStr">
-        <is>
-          <t>AUX-ALOCAR</t>
-        </is>
-      </c>
-      <c r="K66" t="inlineStr">
-        <is>
-          <t>Silvia Ines Coneglian Carrilho de Vasconcelos</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t>2026.2</t>
-        </is>
-      </c>
-      <c r="B67" t="inlineStr">
-        <is>
-          <t>MTM3110</t>
-        </is>
-      </c>
-      <c r="C67" t="inlineStr">
-        <is>
-          <t>01342</t>
-        </is>
-      </c>
-      <c r="D67" t="inlineStr">
-        <is>
-          <t>Cálculo</t>
-        </is>
-      </c>
-      <c r="E67" t="inlineStr">
-        <is>
-          <t>1ª Fase</t>
-        </is>
-      </c>
-      <c r="F67" t="inlineStr">
-        <is>
-          <t>Obrigatória</t>
-        </is>
-      </c>
-      <c r="G67" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="H67" t="inlineStr">
-        <is>
-          <t>72</t>
-        </is>
-      </c>
-      <c r="I67" t="inlineStr">
-        <is>
-          <t>3.1830-2 | 5.1830-2</t>
-        </is>
-      </c>
-      <c r="J67" t="inlineStr">
-        <is>
-          <t>AUX-ALOCAR | AUX-ALOCAR</t>
-        </is>
-      </c>
-      <c r="K67" t="inlineStr">
         <is>
           <t>Francisco Carlos Caramello Junior</t>
         </is>
@@ -7563,12 +7392,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F24"/>
+  <dimension ref="A1:F29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
     <col width="42" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
     <col width="35" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
@@ -7939,17 +7768,17 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>CIN7903 (06342)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>CIN7917 (05342)</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>CIN7904 (06342)</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -7971,17 +7800,17 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>CIN7903 (06342)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>CIN7917 (05342)</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>CIN7904 (06342)</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -7998,12 +7827,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>CIN7945 (05342)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>CIN7938 (05342)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -8030,12 +7859,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>CIN7945 (05342)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>CIN7938 (05342)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -8192,6 +8021,116 @@
       <c r="D24" t="inlineStr">
         <is>
           <t>Nathalia Berger Werlang</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>CIN7903 (06342)</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Inteligência Competitiva</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>AUX-ALOCAR</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>CIN7904 (06342)</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Avaliação de Desempenho</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>AUX-ALOCAR</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Sabrina Borges Ramos de Carvalho</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>CIN7917 (05342)</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Visualização da Informação</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>AUX-ALOCAR</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Márcio Matias</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>CIN7938 (05342)</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Segurança da Informação</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>AUX-ALOCAR</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>CIN7945 (05342)</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Fontes de Informação Tecnológica</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>AUX-ALOCAR</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Márcio Matias</t>
         </is>
       </c>
     </row>
@@ -8210,14 +8149,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="23" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="35" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -8586,7 +8525,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>CIN7905 (05342)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -8596,7 +8535,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>CIN7935 (06342)</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -8618,7 +8557,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>CIN7905 (05342)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -8628,7 +8567,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>CIN7935 (06342)</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -8660,7 +8599,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>CIN7946 (05342)</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -8692,7 +8631,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>CIN7946 (05342)</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -8817,6 +8756,72 @@
       <c r="D23" t="inlineStr">
         <is>
           <t>Márcio Matias</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>CIN7905 (05342)</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Teoria da Decisão</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>AUX-ALOCAR</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Sabrina Borges Ramos de Carvalho</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>CIN7935 (06342)</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Liderança e Gerência</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>CED-LBCON</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Sonali Paula Molin Bedin</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>CIN7946 (05342)</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Pitch de Carreira</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>CED-LBCON</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Sonali Paula Molin Bedin</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
criação de uma nova tabela no supabse "matriz_comun_especifico" para ser acessada pelo banco, e gerar um nova coluna no excel com o nucleo "especifico" ou comun e adicionando os documentos lidos para povoar essa tabela
</commit_message>
<xml_diff>
--- a/resultados/Grade_Horarios_CADASTRO_TURMAS_20262.xlsx
+++ b/resultados/Grade_Horarios_CADASTRO_TURMAS_20262.xlsx
@@ -592,7 +592,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K64"/>
+  <dimension ref="A1:L64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -628,25 +628,30 @@
       </c>
       <c r="G1" t="inlineStr">
         <is>
+          <t>Tipo de Disciplina</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
           <t>Horas Aula</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Ofertas</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Horário</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Local</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Professor</t>
         </is>
@@ -685,25 +690,30 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
+          <t>Comum</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
           <t>72</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>12</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>2.1830-4</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>AUX-ALOCAR</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>Monica Scoz Mendes</t>
         </is>
@@ -742,25 +752,30 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
+          <t>Comum</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
           <t>72</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>12</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>2.1830-4</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>AUX-ALOCAR</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>A contratar</t>
         </is>
@@ -799,25 +814,30 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
+          <t>Comum</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
           <t>36</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>4.1830-2</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>AUX-ALOCAR</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>Ilson Wilmar Rodrigues Filho</t>
         </is>
@@ -856,25 +876,30 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
+          <t>Comum</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
           <t>36</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>20</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>3.2020-2</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>AUX-ALOCAR</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>Sabrina Borges Ramos de Carvalho</t>
         </is>
@@ -913,25 +938,30 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
+          <t>Comum</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
           <t>18</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t>26</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="J6" t="inlineStr">
         <is>
           <t>5.1510-1</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t>AUX-ALOCAR</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="L6" t="inlineStr">
         <is>
           <t>Ricardo Alexandre Reinaldo de Moraes</t>
         </is>
@@ -970,25 +1000,30 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
+          <t>Específico</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
           <t>36</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="I7" t="inlineStr">
         <is>
           <t>28</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="J7" t="inlineStr">
         <is>
           <t>5.1620-2</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="K7" t="inlineStr">
         <is>
           <t>AUX-ALOCAR</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr">
+      <c r="L7" t="inlineStr">
         <is>
           <t>Nathalia Berger Werlang</t>
         </is>
@@ -1027,25 +1062,30 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
+          <t>Comum</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
           <t>72</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="I8" t="inlineStr">
         <is>
           <t>26</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="J8" t="inlineStr">
         <is>
           <t>6.1830-4</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="K8" t="inlineStr">
         <is>
           <t>AUX-ALOCAR</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr">
+      <c r="L8" t="inlineStr">
         <is>
           <t>Mariana Xavier de Oliveira</t>
         </is>
@@ -1084,25 +1124,30 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
+          <t>Comum</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
           <t>18</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="I9" t="inlineStr">
         <is>
           <t>26</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="J9" t="inlineStr">
         <is>
           <t>5.1710-1</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="K9" t="inlineStr">
         <is>
           <t>CED-D109</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr">
+      <c r="L9" t="inlineStr">
         <is>
           <t>Ricardo Alexandre Reinaldo de Moraes</t>
         </is>
@@ -1141,25 +1186,30 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
+          <t>Comum</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
           <t>36</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="I10" t="inlineStr">
         <is>
           <t>12</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="J10" t="inlineStr">
         <is>
           <t>3.1010-2</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="K10" t="inlineStr">
         <is>
           <t>AUX-ALOCAR</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr">
+      <c r="L10" t="inlineStr">
         <is>
           <t>Mariana Xavier de Oliveira</t>
         </is>
@@ -1198,25 +1248,30 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
+          <t>Comum</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
           <t>36</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="I11" t="inlineStr">
         <is>
           <t>12</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
+      <c r="J11" t="inlineStr">
         <is>
           <t>3.2020-2</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="K11" t="inlineStr">
         <is>
           <t>AUX-ALOCAR</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr">
+      <c r="L11" t="inlineStr">
         <is>
           <t>A contratar</t>
         </is>
@@ -1255,25 +1310,30 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
+          <t>Comum</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
           <t>36</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
+      <c r="I12" t="inlineStr">
         <is>
           <t>12</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr">
+      <c r="J12" t="inlineStr">
         <is>
           <t>6.1010-2</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr">
+      <c r="K12" t="inlineStr">
         <is>
           <t>CED-LBPREV</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr">
+      <c r="L12" t="inlineStr">
         <is>
           <t>Maria Zanela</t>
         </is>
@@ -1312,25 +1372,30 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
+          <t>Comum</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
           <t>36</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
+      <c r="I13" t="inlineStr">
         <is>
           <t>12</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr">
+      <c r="J13" t="inlineStr">
         <is>
           <t>5.1830-2</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr">
+      <c r="K13" t="inlineStr">
         <is>
           <t>AUX-ALOCAR</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr">
+      <c r="L13" t="inlineStr">
         <is>
           <t>Edgar Bisset Alvarez</t>
         </is>
@@ -1369,25 +1434,30 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
+          <t>Comum</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
           <t>36</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
+      <c r="I14" t="inlineStr">
         <is>
           <t>12</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr">
+      <c r="J14" t="inlineStr">
         <is>
           <t>2.1010-2</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr">
+      <c r="K14" t="inlineStr">
         <is>
           <t>CED-LBPREV</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr">
+      <c r="L14" t="inlineStr">
         <is>
           <t>Luis Roberto Sousa Mendes</t>
         </is>
@@ -1426,25 +1496,30 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
+          <t>Comum</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
           <t>36</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
+      <c r="I15" t="inlineStr">
         <is>
           <t>12</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr">
+      <c r="J15" t="inlineStr">
         <is>
           <t>2.2020-2</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr">
+      <c r="K15" t="inlineStr">
         <is>
           <t>CED-103 C</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr">
+      <c r="L15" t="inlineStr">
         <is>
           <t>Maria Zanela</t>
         </is>
@@ -1483,25 +1558,30 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
+          <t>Comum</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
           <t>36</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
+      <c r="I16" t="inlineStr">
         <is>
           <t>12</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr">
+      <c r="J16" t="inlineStr">
         <is>
           <t>3.0820-2</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr">
+      <c r="K16" t="inlineStr">
         <is>
           <t>CED-LBTEC</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr">
+      <c r="L16" t="inlineStr">
         <is>
           <t>Gustavo Medeiros de Araújo</t>
         </is>
@@ -1540,25 +1620,30 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
+          <t>Comum</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
           <t>36</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr">
+      <c r="I17" t="inlineStr">
         <is>
           <t>12</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr">
+      <c r="J17" t="inlineStr">
         <is>
           <t>5.2020-2</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr">
+      <c r="K17" t="inlineStr">
         <is>
           <t>CED-102 C</t>
         </is>
       </c>
-      <c r="K17" t="inlineStr">
+      <c r="L17" t="inlineStr">
         <is>
           <t>Gustavo Medeiros de Araújo</t>
         </is>
@@ -1597,25 +1682,30 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
+          <t>Comum</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
           <t>36</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr">
+      <c r="I18" t="inlineStr">
         <is>
           <t>12</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr">
+      <c r="J18" t="inlineStr">
         <is>
           <t>6.0820-2</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr">
+      <c r="K18" t="inlineStr">
         <is>
           <t>CED-LBPREV</t>
         </is>
       </c>
-      <c r="K18" t="inlineStr">
+      <c r="L18" t="inlineStr">
         <is>
           <t>Maria Zanela</t>
         </is>
@@ -1654,25 +1744,30 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
+          <t>Comum</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
           <t>36</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr">
+      <c r="I19" t="inlineStr">
         <is>
           <t>12</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr">
+      <c r="J19" t="inlineStr">
         <is>
           <t>2.1830-2</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr">
+      <c r="K19" t="inlineStr">
         <is>
           <t>CED-103 C</t>
         </is>
       </c>
-      <c r="K19" t="inlineStr">
+      <c r="L19" t="inlineStr">
         <is>
           <t>Maria Zanela</t>
         </is>
@@ -1711,25 +1806,30 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
+          <t>Comum</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
           <t>72</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr">
+      <c r="I20" t="inlineStr">
         <is>
           <t>24</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr">
+      <c r="J20" t="inlineStr">
         <is>
           <t>4.1830-4</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr">
+      <c r="K20" t="inlineStr">
         <is>
           <t>CED-LBTEC</t>
         </is>
       </c>
-      <c r="K20" t="inlineStr">
+      <c r="L20" t="inlineStr">
         <is>
           <t>A contratar</t>
         </is>
@@ -1768,25 +1868,30 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
+          <t>Comum</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
           <t>72</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr">
+      <c r="I21" t="inlineStr">
         <is>
           <t>24</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr">
+      <c r="J21" t="inlineStr">
         <is>
           <t>4.0820-4</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr">
+      <c r="K21" t="inlineStr">
         <is>
           <t>CED-LBTEC</t>
         </is>
       </c>
-      <c r="K21" t="inlineStr">
+      <c r="L21" t="inlineStr">
         <is>
           <t>A contratar</t>
         </is>
@@ -1825,25 +1930,30 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
+          <t>Comum</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
           <t>72</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr">
+      <c r="I22" t="inlineStr">
         <is>
           <t>12</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr">
+      <c r="J22" t="inlineStr">
         <is>
           <t>2.0820-4</t>
         </is>
       </c>
-      <c r="J22" t="inlineStr">
+      <c r="K22" t="inlineStr">
         <is>
           <t>CED-103 C</t>
         </is>
       </c>
-      <c r="K22" t="inlineStr">
+      <c r="L22" t="inlineStr">
         <is>
           <t>Adilson Luiz Pinto</t>
         </is>
@@ -1882,25 +1992,30 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
+          <t>Comum</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
           <t>72</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr">
+      <c r="I23" t="inlineStr">
         <is>
           <t>12</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr">
+      <c r="J23" t="inlineStr">
         <is>
           <t>3.1830-4</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr">
+      <c r="K23" t="inlineStr">
         <is>
           <t>CED-103 C</t>
         </is>
       </c>
-      <c r="K23" t="inlineStr">
+      <c r="L23" t="inlineStr">
         <is>
           <t>Adilson Luiz Pinto</t>
         </is>
@@ -1939,25 +2054,30 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
+          <t>Comum</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
           <t>36</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr">
+      <c r="I24" t="inlineStr">
         <is>
           <t>12</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr">
+      <c r="J24" t="inlineStr">
         <is>
           <t>6.1010-2</t>
         </is>
       </c>
-      <c r="J24" t="inlineStr">
+      <c r="K24" t="inlineStr">
         <is>
           <t>CED-LBTEC</t>
         </is>
       </c>
-      <c r="K24" t="inlineStr">
+      <c r="L24" t="inlineStr">
         <is>
           <t>Enrique Muriel Torrado</t>
         </is>
@@ -1996,25 +2116,30 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
+          <t>Comum</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
           <t>36</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr">
+      <c r="I25" t="inlineStr">
         <is>
           <t>12</t>
         </is>
       </c>
-      <c r="I25" t="inlineStr">
+      <c r="J25" t="inlineStr">
         <is>
           <t>6.1830-2</t>
         </is>
       </c>
-      <c r="J25" t="inlineStr">
+      <c r="K25" t="inlineStr">
         <is>
           <t>CED-103 C</t>
         </is>
       </c>
-      <c r="K25" t="inlineStr">
+      <c r="L25" t="inlineStr">
         <is>
           <t>Enrique Muriel Torrado</t>
         </is>
@@ -2053,25 +2178,30 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
+          <t>Comum</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
           <t>36</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr">
+      <c r="I26" t="inlineStr">
         <is>
           <t>24</t>
         </is>
       </c>
-      <c r="I26" t="inlineStr">
+      <c r="J26" t="inlineStr">
         <is>
           <t>2.1710-1 | 4.1710-1</t>
         </is>
       </c>
-      <c r="J26" t="inlineStr">
+      <c r="K26" t="inlineStr">
         <is>
           <t>CED-LBPREV | CED-LBPREV</t>
         </is>
       </c>
-      <c r="K26" t="inlineStr">
+      <c r="L26" t="inlineStr">
         <is>
           <t>Ilson Wilmar Rodrigues Filho</t>
         </is>
@@ -2110,25 +2240,30 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
+          <t>Comum</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
           <t>36</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr">
+      <c r="I27" t="inlineStr">
         <is>
           <t>12</t>
         </is>
       </c>
-      <c r="I27" t="inlineStr">
+      <c r="J27" t="inlineStr">
         <is>
           <t>4.0730-1 | 6.0730-1</t>
         </is>
       </c>
-      <c r="J27" t="inlineStr">
+      <c r="K27" t="inlineStr">
         <is>
           <t>CED-103 C | CED-103 C</t>
         </is>
       </c>
-      <c r="K27" t="inlineStr">
+      <c r="L27" t="inlineStr">
         <is>
           <t>Maria Zanela</t>
         </is>
@@ -2167,25 +2302,30 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
+          <t>Comum</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
           <t>36</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr">
+      <c r="I28" t="inlineStr">
         <is>
           <t>12</t>
         </is>
       </c>
-      <c r="I28" t="inlineStr">
+      <c r="J28" t="inlineStr">
         <is>
           <t>6.2020-2</t>
         </is>
       </c>
-      <c r="J28" t="inlineStr">
+      <c r="K28" t="inlineStr">
         <is>
           <t>CED-LBTEC</t>
         </is>
       </c>
-      <c r="K28" t="inlineStr">
+      <c r="L28" t="inlineStr">
         <is>
           <t>Sabrina Borges Ramos de Carvalho</t>
         </is>
@@ -2224,25 +2364,30 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
+          <t>Comum</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
           <t>36</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr">
+      <c r="I29" t="inlineStr">
         <is>
           <t>12</t>
         </is>
       </c>
-      <c r="I29" t="inlineStr">
+      <c r="J29" t="inlineStr">
         <is>
           <t>5.1010-2</t>
         </is>
       </c>
-      <c r="J29" t="inlineStr">
+      <c r="K29" t="inlineStr">
         <is>
           <t>CED-LBTEC</t>
         </is>
       </c>
-      <c r="K29" t="inlineStr">
+      <c r="L29" t="inlineStr">
         <is>
           <t>Flavio Augusto Carraro</t>
         </is>
@@ -2281,25 +2426,30 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
+          <t>Comum</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
           <t>36</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr">
+      <c r="I30" t="inlineStr">
         <is>
           <t>12</t>
         </is>
       </c>
-      <c r="I30" t="inlineStr">
+      <c r="J30" t="inlineStr">
         <is>
           <t>4.2020-2</t>
         </is>
       </c>
-      <c r="J30" t="inlineStr">
+      <c r="K30" t="inlineStr">
         <is>
           <t>CED-LBPREV</t>
         </is>
       </c>
-      <c r="K30" t="inlineStr">
+      <c r="L30" t="inlineStr">
         <is>
           <t>Flavio Augusto Carraro</t>
         </is>
@@ -2338,25 +2488,30 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
+          <t>Comum</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
           <t>36</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr">
+      <c r="I31" t="inlineStr">
         <is>
           <t>12</t>
         </is>
       </c>
-      <c r="I31" t="inlineStr">
+      <c r="J31" t="inlineStr">
         <is>
           <t>6.0820-2</t>
         </is>
       </c>
-      <c r="J31" t="inlineStr">
+      <c r="K31" t="inlineStr">
         <is>
           <t>CED-LBTEC</t>
         </is>
       </c>
-      <c r="K31" t="inlineStr">
+      <c r="L31" t="inlineStr">
         <is>
           <t>Enrique Muriel Torrado</t>
         </is>
@@ -2395,25 +2550,30 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
+          <t>Comum</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
           <t>36</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr">
+      <c r="I32" t="inlineStr">
         <is>
           <t>12</t>
         </is>
       </c>
-      <c r="I32" t="inlineStr">
+      <c r="J32" t="inlineStr">
         <is>
           <t>2.2020-2</t>
         </is>
       </c>
-      <c r="J32" t="inlineStr">
+      <c r="K32" t="inlineStr">
         <is>
           <t>CED-LBPREV</t>
         </is>
       </c>
-      <c r="K32" t="inlineStr">
+      <c r="L32" t="inlineStr">
         <is>
           <t>Sabrina Borges Ramos de Carvalho</t>
         </is>
@@ -2452,25 +2612,30 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
+          <t>Comum</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
           <t>36</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr">
+      <c r="I33" t="inlineStr">
         <is>
           <t>24</t>
         </is>
       </c>
-      <c r="I33" t="inlineStr">
+      <c r="J33" t="inlineStr">
         <is>
           <t>5.2020-2</t>
         </is>
       </c>
-      <c r="J33" t="inlineStr">
+      <c r="K33" t="inlineStr">
         <is>
           <t>AUX-ALOCAR</t>
         </is>
       </c>
-      <c r="K33" t="inlineStr">
+      <c r="L33" t="inlineStr">
         <is>
           <t>Sabrina Borges Ramos de Carvalho</t>
         </is>
@@ -2509,25 +2674,30 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
+          <t>Comum</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
           <t>36</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr">
+      <c r="I34" t="inlineStr">
         <is>
           <t>24</t>
         </is>
       </c>
-      <c r="I34" t="inlineStr">
+      <c r="J34" t="inlineStr">
         <is>
           <t>3.1010-2</t>
         </is>
       </c>
-      <c r="J34" t="inlineStr">
+      <c r="K34" t="inlineStr">
         <is>
           <t>CED-004 D</t>
         </is>
       </c>
-      <c r="K34" t="inlineStr">
+      <c r="L34" t="inlineStr">
         <is>
           <t>Sonali Paula Molin Bedin</t>
         </is>
@@ -2566,25 +2736,30 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
+          <t>Específico</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
           <t>36</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr">
+      <c r="I35" t="inlineStr">
         <is>
           <t>26</t>
         </is>
       </c>
-      <c r="I35" t="inlineStr">
+      <c r="J35" t="inlineStr">
         <is>
           <t>2.1830-2</t>
         </is>
       </c>
-      <c r="J35" t="inlineStr">
+      <c r="K35" t="inlineStr">
         <is>
           <t>AUX-ALOCAR</t>
         </is>
       </c>
-      <c r="K35" t="inlineStr">
+      <c r="L35" t="inlineStr">
         <is>
           <t>Márcio Matias</t>
         </is>
@@ -2623,25 +2798,30 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
+          <t>Específico</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
           <t>36</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr">
+      <c r="I36" t="inlineStr">
         <is>
           <t>26</t>
         </is>
       </c>
-      <c r="I36" t="inlineStr">
+      <c r="J36" t="inlineStr">
         <is>
           <t>5.2020-2</t>
         </is>
       </c>
-      <c r="J36" t="inlineStr">
+      <c r="K36" t="inlineStr">
         <is>
           <t>AUX-ALOCAR</t>
         </is>
       </c>
-      <c r="K36" t="inlineStr">
+      <c r="L36" t="inlineStr">
         <is>
           <t>Flavio Augusto Carraro</t>
         </is>
@@ -2680,25 +2860,30 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
+          <t>Específico</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
           <t>36</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr">
+      <c r="I37" t="inlineStr">
         <is>
           <t>26</t>
         </is>
       </c>
-      <c r="I37" t="inlineStr">
+      <c r="J37" t="inlineStr">
         <is>
           <t>6.2020-2</t>
         </is>
       </c>
-      <c r="J37" t="inlineStr">
+      <c r="K37" t="inlineStr">
         <is>
           <t>AUX-ALOCAR</t>
         </is>
       </c>
-      <c r="K37" t="inlineStr">
+      <c r="L37" t="inlineStr">
         <is>
           <t>Flavio Augusto Carraro</t>
         </is>
@@ -2737,25 +2922,30 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
+          <t>Específico</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
           <t>36</t>
         </is>
       </c>
-      <c r="H38" t="inlineStr">
+      <c r="I38" t="inlineStr">
         <is>
           <t>26</t>
         </is>
       </c>
-      <c r="I38" t="inlineStr">
+      <c r="J38" t="inlineStr">
         <is>
           <t>6.1830-2</t>
         </is>
       </c>
-      <c r="J38" t="inlineStr">
+      <c r="K38" t="inlineStr">
         <is>
           <t>AUX-ALOCAR</t>
         </is>
       </c>
-      <c r="K38" t="inlineStr">
+      <c r="L38" t="inlineStr">
         <is>
           <t>Sabrina Borges Ramos de Carvalho</t>
         </is>
@@ -2794,25 +2984,30 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
+          <t>Específico</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
           <t>432</t>
         </is>
       </c>
-      <c r="H39" t="inlineStr">
+      <c r="I39" t="inlineStr">
         <is>
           <t>26</t>
         </is>
       </c>
-      <c r="I39" t="inlineStr">
+      <c r="J39" t="inlineStr">
         <is>
           <t>2.1420-2</t>
         </is>
       </c>
-      <c r="J39" t="inlineStr">
+      <c r="K39" t="inlineStr">
         <is>
           <t>CED-105 B</t>
         </is>
       </c>
-      <c r="K39" t="inlineStr">
+      <c r="L39" t="inlineStr">
         <is>
           <t>Nathalia Berger Werlang</t>
         </is>
@@ -2851,25 +3046,30 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
+          <t>Específico</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
           <t>36</t>
         </is>
       </c>
-      <c r="H40" t="inlineStr">
+      <c r="I40" t="inlineStr">
         <is>
           <t>26</t>
         </is>
       </c>
-      <c r="I40" t="inlineStr">
+      <c r="J40" t="inlineStr">
         <is>
           <t>4.1830-2</t>
         </is>
       </c>
-      <c r="J40" t="inlineStr">
+      <c r="K40" t="inlineStr">
         <is>
           <t>AUX-ALOCAR</t>
         </is>
       </c>
-      <c r="K40" t="inlineStr">
+      <c r="L40" t="inlineStr">
         <is>
           <t>Flavio Augusto Carraro</t>
         </is>
@@ -2908,25 +3108,30 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
+          <t>Específico</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
           <t>36</t>
         </is>
       </c>
-      <c r="H41" t="inlineStr">
+      <c r="I41" t="inlineStr">
         <is>
           <t>26</t>
         </is>
       </c>
-      <c r="I41" t="inlineStr">
+      <c r="J41" t="inlineStr">
         <is>
           <t>6.1830-2</t>
         </is>
       </c>
-      <c r="J41" t="inlineStr">
+      <c r="K41" t="inlineStr">
         <is>
           <t>AUX-ALOCAR</t>
         </is>
       </c>
-      <c r="K41" t="inlineStr">
+      <c r="L41" t="inlineStr">
         <is>
           <t>Flavio Augusto Carraro</t>
         </is>
@@ -2965,25 +3170,30 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
+          <t>Específico</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
           <t>72</t>
         </is>
       </c>
-      <c r="H42" t="inlineStr">
+      <c r="I42" t="inlineStr">
         <is>
           <t>26</t>
         </is>
       </c>
-      <c r="I42" t="inlineStr">
+      <c r="J42" t="inlineStr">
         <is>
           <t>2.1830-4</t>
         </is>
       </c>
-      <c r="J42" t="inlineStr">
+      <c r="K42" t="inlineStr">
         <is>
           <t>AUX-ALOCAR</t>
         </is>
       </c>
-      <c r="K42" t="inlineStr">
+      <c r="L42" t="inlineStr">
         <is>
           <t>Nathalia Berger Werlang</t>
         </is>
@@ -3022,25 +3232,30 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
+          <t>Específico</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
           <t>74</t>
         </is>
       </c>
-      <c r="H43" t="inlineStr">
+      <c r="I43" t="inlineStr">
         <is>
           <t>26</t>
         </is>
       </c>
-      <c r="I43" t="inlineStr">
+      <c r="J43" t="inlineStr">
         <is>
           <t>4.1620-2</t>
         </is>
       </c>
-      <c r="J43" t="inlineStr">
+      <c r="K43" t="inlineStr">
         <is>
           <t>AUX-ALOCAR</t>
         </is>
       </c>
-      <c r="K43" t="inlineStr">
+      <c r="L43" t="inlineStr">
         <is>
           <t>Márcio Matias</t>
         </is>
@@ -3079,25 +3294,30 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
+          <t>Específico</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
           <t>36</t>
         </is>
       </c>
-      <c r="H44" t="inlineStr">
+      <c r="I44" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="I44" t="inlineStr">
+      <c r="J44" t="inlineStr">
         <is>
           <t>3.1830-2</t>
         </is>
       </c>
-      <c r="J44" t="inlineStr">
+      <c r="K44" t="inlineStr">
         <is>
           <t>AUX-ALOCAR</t>
         </is>
       </c>
-      <c r="K44" t="inlineStr">
+      <c r="L44" t="inlineStr">
         <is>
           <t>A contratar</t>
         </is>
@@ -3136,25 +3356,30 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
+          <t>Comum</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
           <t>36</t>
         </is>
       </c>
-      <c r="H45" t="inlineStr">
+      <c r="I45" t="inlineStr">
         <is>
           <t>26</t>
         </is>
       </c>
-      <c r="I45" t="inlineStr">
+      <c r="J45" t="inlineStr">
         <is>
           <t>5.1830-2</t>
         </is>
       </c>
-      <c r="J45" t="inlineStr">
+      <c r="K45" t="inlineStr">
         <is>
           <t>AUX-ALOCAR</t>
         </is>
       </c>
-      <c r="K45" t="inlineStr">
+      <c r="L45" t="inlineStr">
         <is>
           <t>Sabrina Borges Ramos de Carvalho</t>
         </is>
@@ -3193,25 +3418,30 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
+          <t>Comum</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
           <t>36</t>
         </is>
       </c>
-      <c r="H46" t="inlineStr">
+      <c r="I46" t="inlineStr">
         <is>
           <t>26</t>
         </is>
       </c>
-      <c r="I46" t="inlineStr">
+      <c r="J46" t="inlineStr">
         <is>
           <t>3.1830-2</t>
         </is>
       </c>
-      <c r="J46" t="inlineStr">
+      <c r="K46" t="inlineStr">
         <is>
           <t>AUX-ALOCAR</t>
         </is>
       </c>
-      <c r="K46" t="inlineStr">
+      <c r="L46" t="inlineStr">
         <is>
           <t>Sabrina Borges Ramos de Carvalho</t>
         </is>
@@ -3250,25 +3480,30 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
+          <t>Específico</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
           <t>72</t>
         </is>
       </c>
-      <c r="H47" t="inlineStr">
+      <c r="I47" t="inlineStr">
         <is>
           <t>26</t>
         </is>
       </c>
-      <c r="I47" t="inlineStr">
+      <c r="J47" t="inlineStr">
         <is>
           <t>3.1830-4</t>
         </is>
       </c>
-      <c r="J47" t="inlineStr">
+      <c r="K47" t="inlineStr">
         <is>
           <t>AUX-ALOCAR</t>
         </is>
       </c>
-      <c r="K47" t="inlineStr">
+      <c r="L47" t="inlineStr">
         <is>
           <t>Flavio Augusto Carraro</t>
         </is>
@@ -3307,25 +3542,30 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
+          <t>Comum</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
           <t>36</t>
         </is>
       </c>
-      <c r="H48" t="inlineStr">
+      <c r="I48" t="inlineStr">
         <is>
           <t>26</t>
         </is>
       </c>
-      <c r="I48" t="inlineStr">
+      <c r="J48" t="inlineStr">
         <is>
           <t>4.1830-2</t>
         </is>
       </c>
-      <c r="J48" t="inlineStr">
+      <c r="K48" t="inlineStr">
         <is>
           <t>AUX-ALOCAR</t>
         </is>
       </c>
-      <c r="K48" t="inlineStr">
+      <c r="L48" t="inlineStr">
         <is>
           <t>Márcio Matias</t>
         </is>
@@ -3364,25 +3604,30 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
+          <t>Comum</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
           <t>36</t>
         </is>
       </c>
-      <c r="H49" t="inlineStr">
+      <c r="I49" t="inlineStr">
         <is>
           <t>26</t>
         </is>
       </c>
-      <c r="I49" t="inlineStr">
+      <c r="J49" t="inlineStr">
         <is>
           <t>5.2020-2</t>
         </is>
       </c>
-      <c r="J49" t="inlineStr">
+      <c r="K49" t="inlineStr">
         <is>
           <t>AUX-ALOCAR</t>
         </is>
       </c>
-      <c r="K49" t="inlineStr">
+      <c r="L49" t="inlineStr">
         <is>
           <t>Ricardo Alexandre Reinaldo de Moraes</t>
         </is>
@@ -3421,25 +3666,30 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
+          <t>Comum</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
           <t>36</t>
         </is>
       </c>
-      <c r="H50" t="inlineStr">
+      <c r="I50" t="inlineStr">
         <is>
           <t>26</t>
         </is>
       </c>
-      <c r="I50" t="inlineStr">
+      <c r="J50" t="inlineStr">
         <is>
           <t>2.1830-2</t>
         </is>
       </c>
-      <c r="J50" t="inlineStr">
+      <c r="K50" t="inlineStr">
         <is>
           <t>AUX-ALOCAR</t>
         </is>
       </c>
-      <c r="K50" t="inlineStr">
+      <c r="L50" t="inlineStr">
         <is>
           <t>Sabrina Borges Ramos de Carvalho</t>
         </is>
@@ -3478,25 +3728,30 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
+          <t>Comum</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
           <t>36</t>
         </is>
       </c>
-      <c r="H51" t="inlineStr">
+      <c r="I51" t="inlineStr">
         <is>
           <t>26</t>
         </is>
       </c>
-      <c r="I51" t="inlineStr">
+      <c r="J51" t="inlineStr">
         <is>
           <t>5.1830-2</t>
         </is>
       </c>
-      <c r="J51" t="inlineStr">
+      <c r="K51" t="inlineStr">
         <is>
           <t>CED-LBCON</t>
         </is>
       </c>
-      <c r="K51" t="inlineStr">
+      <c r="L51" t="inlineStr">
         <is>
           <t>Sonali Paula Molin Bedin</t>
         </is>
@@ -3535,25 +3790,30 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
+          <t>Comum</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
           <t>36</t>
         </is>
       </c>
-      <c r="H52" t="inlineStr">
+      <c r="I52" t="inlineStr">
         <is>
           <t>12</t>
         </is>
       </c>
-      <c r="I52" t="inlineStr">
+      <c r="J52" t="inlineStr">
         <is>
           <t>2.0820-2</t>
         </is>
       </c>
-      <c r="J52" t="inlineStr">
+      <c r="K52" t="inlineStr">
         <is>
           <t>CED-LBPREV</t>
         </is>
       </c>
-      <c r="K52" t="inlineStr">
+      <c r="L52" t="inlineStr">
         <is>
           <t>Marcelo Minghelli</t>
         </is>
@@ -3592,25 +3852,30 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
+          <t>Comum</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
           <t>36</t>
         </is>
       </c>
-      <c r="H53" t="inlineStr">
+      <c r="I53" t="inlineStr">
         <is>
           <t>12</t>
         </is>
       </c>
-      <c r="I53" t="inlineStr">
+      <c r="J53" t="inlineStr">
         <is>
           <t>3.1830-2</t>
         </is>
       </c>
-      <c r="J53" t="inlineStr">
+      <c r="K53" t="inlineStr">
         <is>
           <t>CED-102 C</t>
         </is>
       </c>
-      <c r="K53" t="inlineStr">
+      <c r="L53" t="inlineStr">
         <is>
           <t>Marcelo Minghelli</t>
         </is>
@@ -3649,25 +3914,30 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
+          <t>Específico</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
           <t>36</t>
         </is>
       </c>
-      <c r="H54" t="inlineStr">
+      <c r="I54" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="I54" t="inlineStr">
+      <c r="J54" t="inlineStr">
         <is>
           <t>3.2020-2</t>
         </is>
       </c>
-      <c r="J54" t="inlineStr">
+      <c r="K54" t="inlineStr">
         <is>
           <t>AUX-ALOCAR</t>
         </is>
       </c>
-      <c r="K54" t="inlineStr">
+      <c r="L54" t="inlineStr">
         <is>
           <t>A contratar</t>
         </is>
@@ -3706,25 +3976,30 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
+          <t>Específico</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
           <t>36</t>
         </is>
       </c>
-      <c r="H55" t="inlineStr">
+      <c r="I55" t="inlineStr">
         <is>
           <t>26</t>
         </is>
       </c>
-      <c r="I55" t="inlineStr">
+      <c r="J55" t="inlineStr">
         <is>
           <t>4.2020-2</t>
         </is>
       </c>
-      <c r="J55" t="inlineStr">
+      <c r="K55" t="inlineStr">
         <is>
           <t>AUX-ALOCAR</t>
         </is>
       </c>
-      <c r="K55" t="inlineStr">
+      <c r="L55" t="inlineStr">
         <is>
           <t>Márcio Matias</t>
         </is>
@@ -3763,25 +4038,30 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
+          <t>Específico</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
           <t>36</t>
         </is>
       </c>
-      <c r="H56" t="inlineStr">
+      <c r="I56" t="inlineStr">
         <is>
           <t>26</t>
         </is>
       </c>
-      <c r="I56" t="inlineStr">
+      <c r="J56" t="inlineStr">
         <is>
           <t>2.2020-2</t>
         </is>
       </c>
-      <c r="J56" t="inlineStr">
+      <c r="K56" t="inlineStr">
         <is>
           <t>AUX-ALOCAR</t>
         </is>
       </c>
-      <c r="K56" t="inlineStr">
+      <c r="L56" t="inlineStr">
         <is>
           <t>Márcio Matias</t>
         </is>
@@ -3820,25 +4100,30 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
+          <t>Específico</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
           <t>36</t>
         </is>
       </c>
-      <c r="H57" t="inlineStr">
+      <c r="I57" t="inlineStr">
         <is>
           <t>26</t>
         </is>
       </c>
-      <c r="I57" t="inlineStr">
+      <c r="J57" t="inlineStr">
         <is>
           <t>5.2020-2</t>
         </is>
       </c>
-      <c r="J57" t="inlineStr">
+      <c r="K57" t="inlineStr">
         <is>
           <t>CED-LBCON</t>
         </is>
       </c>
-      <c r="K57" t="inlineStr">
+      <c r="L57" t="inlineStr">
         <is>
           <t>Sonali Paula Molin Bedin</t>
         </is>
@@ -3877,25 +4162,30 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
+          <t>Comum</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
           <t>72</t>
         </is>
       </c>
-      <c r="H58" t="inlineStr">
+      <c r="I58" t="inlineStr">
         <is>
           <t>12</t>
         </is>
       </c>
-      <c r="I58" t="inlineStr">
+      <c r="J58" t="inlineStr">
         <is>
           <t>5.0820-4</t>
         </is>
       </c>
-      <c r="J58" t="inlineStr">
+      <c r="K58" t="inlineStr">
         <is>
           <t>CED-LBPREV</t>
         </is>
       </c>
-      <c r="K58" t="inlineStr">
+      <c r="L58" t="inlineStr">
         <is>
           <t>Roselane Neckel</t>
         </is>
@@ -3934,25 +4224,30 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
+          <t>Comum</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
           <t>72</t>
         </is>
       </c>
-      <c r="H59" t="inlineStr">
+      <c r="I59" t="inlineStr">
         <is>
           <t>12</t>
         </is>
       </c>
-      <c r="I59" t="inlineStr">
+      <c r="J59" t="inlineStr">
         <is>
           <t>6.1830-4</t>
         </is>
       </c>
-      <c r="J59" t="inlineStr">
+      <c r="K59" t="inlineStr">
         <is>
           <t>CED-LBPREV</t>
         </is>
       </c>
-      <c r="K59" t="inlineStr">
+      <c r="L59" t="inlineStr">
         <is>
           <t>Roselane Neckel</t>
         </is>
@@ -3991,25 +4286,30 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
+          <t>Comum</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
           <t>72</t>
         </is>
       </c>
-      <c r="H60" t="inlineStr">
+      <c r="I60" t="inlineStr">
         <is>
           <t>24</t>
         </is>
       </c>
-      <c r="I60" t="inlineStr">
+      <c r="J60" t="inlineStr">
         <is>
           <t>3.0820-2 | 4.1010-2</t>
         </is>
       </c>
-      <c r="J60" t="inlineStr">
+      <c r="K60" t="inlineStr">
         <is>
           <t>CED-LBPREV | CED-LBPREV</t>
         </is>
       </c>
-      <c r="K60" t="inlineStr">
+      <c r="L60" t="inlineStr">
         <is>
           <t>Vera do Carmo Comparsi de Vargas</t>
         </is>
@@ -4048,25 +4348,30 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
+          <t>Comum</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
           <t>72</t>
         </is>
       </c>
-      <c r="H61" t="inlineStr">
+      <c r="I61" t="inlineStr">
         <is>
           <t>24</t>
         </is>
       </c>
-      <c r="I61" t="inlineStr">
+      <c r="J61" t="inlineStr">
         <is>
           <t>2.1830-2 | 5.1830-2</t>
         </is>
       </c>
-      <c r="J61" t="inlineStr">
+      <c r="K61" t="inlineStr">
         <is>
           <t>CED-LBPREV | CED-102 C</t>
         </is>
       </c>
-      <c r="K61" t="inlineStr">
+      <c r="L61" t="inlineStr">
         <is>
           <t>Manoella Reis Cardenuto</t>
         </is>
@@ -4105,25 +4410,30 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
+          <t>Comum</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
           <t>72</t>
         </is>
       </c>
-      <c r="H62" t="inlineStr">
+      <c r="I62" t="inlineStr">
         <is>
           <t>12</t>
         </is>
       </c>
-      <c r="I62" t="inlineStr">
+      <c r="J62" t="inlineStr">
         <is>
           <t>6.1830-4</t>
         </is>
       </c>
-      <c r="J62" t="inlineStr">
+      <c r="K62" t="inlineStr">
         <is>
           <t>AUX-ALOCAR</t>
         </is>
       </c>
-      <c r="K62" t="inlineStr">
+      <c r="L62" t="inlineStr">
         <is>
           <t>Gabriela Rempel</t>
         </is>
@@ -4162,25 +4472,30 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
+          <t>Comum</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
           <t>72</t>
         </is>
       </c>
-      <c r="H63" t="inlineStr">
+      <c r="I63" t="inlineStr">
         <is>
           <t>12</t>
         </is>
       </c>
-      <c r="I63" t="inlineStr">
+      <c r="J63" t="inlineStr">
         <is>
           <t>6.1830-4</t>
         </is>
       </c>
-      <c r="J63" t="inlineStr">
+      <c r="K63" t="inlineStr">
         <is>
           <t>AUX-ALOCAR</t>
         </is>
       </c>
-      <c r="K63" t="inlineStr">
+      <c r="L63" t="inlineStr">
         <is>
           <t>Silvia Ines Coneglian Carrilho de Vasconcelos</t>
         </is>
@@ -4219,25 +4534,30 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
+          <t>Específico</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="H64" t="inlineStr">
+      <c r="I64" t="inlineStr">
         <is>
           <t>72</t>
         </is>
       </c>
-      <c r="I64" t="inlineStr">
+      <c r="J64" t="inlineStr">
         <is>
           <t>3.1830-2 | 5.1830-2</t>
         </is>
       </c>
-      <c r="J64" t="inlineStr">
+      <c r="K64" t="inlineStr">
         <is>
           <t>AUX-ALOCAR | AUX-ALOCAR</t>
         </is>
       </c>
-      <c r="K64" t="inlineStr">
+      <c r="L64" t="inlineStr">
         <is>
           <t>Francisco Carlos Caramello Junior</t>
         </is>

</xml_diff>